<commit_message>
fix(#106): synchronize reviewed financial and navigation corrections
</commit_message>
<xml_diff>
--- a/docs/research/integrated-product-106/Experience/cases/HOME-12/HOME-12_Evidence_Workbook.xlsx
+++ b/docs/research/integrated-product-106/Experience/cases/HOME-12/HOME-12_Evidence_Workbook.xlsx
@@ -15,13 +15,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurement" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'START HERE'!$A$1:$L$44</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'START HERE'!$A$1:$L$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Findings'!$A$1:$D$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Findings'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Findings'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Owner WBS'!$A$1:$C$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Owner WBS'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Owner WBS'!$A$1:$C$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Owner WBS'!$A$1:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Crosswalk'!$A$1:$N$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Crosswalk'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Crosswalk'!$B$1:$N$11</definedName>
@@ -167,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -243,6 +243,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -384,7 +387,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr sz="1100" b="0">
                 <a:latin typeface="Archivo"/>
@@ -435,7 +438,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr sz="1100" b="0">
               <a:latin typeface="Archivo"/>
@@ -463,7 +466,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr sz="1100" b="0">
               <a:latin typeface="Archivo"/>
@@ -543,7 +546,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t/>
+                <a:t>None</a:t>
               </a:r>
               <a:endParaRPr sz="1100" b="0">
                 <a:latin typeface="Archivo"/>
@@ -594,7 +597,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr sz="1100" b="0">
               <a:latin typeface="Archivo"/>
@@ -622,7 +625,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr sz="1100" b="0">
               <a:latin typeface="Archivo"/>
@@ -1149,8 +1152,38 @@
     <row r="42" ht="19" customHeight="1"/>
     <row r="43" ht="19" customHeight="1"/>
     <row r="44" ht="19" customHeight="1"/>
-    <row r="45" ht="19" customHeight="1"/>
-    <row r="46" ht="19" customHeight="1"/>
+    <row r="45" ht="19" customHeight="1">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>Counting, authority and measurement →</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="8" t="n"/>
+      <c r="E45" s="8" t="n"/>
+      <c r="F45" s="8" t="n"/>
+      <c r="G45" s="8" t="n"/>
+      <c r="H45" s="8" t="n"/>
+      <c r="I45" s="8" t="n"/>
+      <c r="J45" s="8" t="n"/>
+      <c r="K45" s="8" t="n"/>
+      <c r="L45" s="8" t="n"/>
+    </row>
+    <row r="46" ht="19" customHeight="1">
+      <c r="A46" s="8" t="n"/>
+      <c r="B46" s="8" t="n"/>
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="8" t="n"/>
+      <c r="E46" s="8" t="n"/>
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="8" t="n"/>
+      <c r="H46" s="8" t="n"/>
+      <c r="I46" s="8" t="n"/>
+      <c r="J46" s="8" t="n"/>
+      <c r="K46" s="8" t="n"/>
+      <c r="L46" s="8" t="n"/>
+    </row>
     <row r="47" ht="19" customHeight="1">
       <c r="A47" t="inlineStr">
         <is>
@@ -1301,7 +1334,7 @@
     <row r="78" ht="19" customHeight="1"/>
     <row r="79" ht="19" customHeight="1"/>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="30">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A12:D14"/>
     <mergeCell ref="A24:D25"/>
@@ -1319,6 +1352,7 @@
     <mergeCell ref="I11:L11"/>
     <mergeCell ref="E5:H5"/>
     <mergeCell ref="D51:F51"/>
+    <mergeCell ref="A45:L46"/>
     <mergeCell ref="A10:L10"/>
     <mergeCell ref="A20:L22"/>
     <mergeCell ref="D54:F54"/>
@@ -1336,6 +1370,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId4"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>
@@ -1351,7 +1386,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="26" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
 </worksheet>
 </file>
 
@@ -1508,12 +1543,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1532,9 +1568,14 @@
           <t>Parent</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="35" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Related source route / Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="45" customHeight="1">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>H12</t>
         </is>
@@ -1545,9 +1586,14 @@
         </is>
       </c>
       <c r="C2" s="24" t="inlineStr"/>
-    </row>
-    <row r="3" ht="35" customHeight="1">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>Inspect first related source record →</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>H12.10</t>
         </is>
@@ -1562,9 +1608,14 @@
           <t>H12</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="35" customHeight="1">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Inspect first related source record →</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="45" customHeight="1">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>H12.20</t>
         </is>
@@ -1579,9 +1630,14 @@
           <t>H12</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="35" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Inspect first related source record →</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="45" customHeight="1">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>H12.30</t>
         </is>
@@ -1596,8 +1652,13 @@
           <t>H12</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="35" customHeight="1">
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>Inspect first related source record →</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="24" t="inlineStr">
         <is>
           <t>H12.40</t>
@@ -1611,6 +1672,11 @@
       <c r="C6" s="24" t="inlineStr">
         <is>
           <t>H12</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>No related source record supplied. Missing is not zero.</t>
         </is>
       </c>
     </row>
@@ -1618,11 +1684,15 @@
   <autoFilter ref="A1:C6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
fix(#106): synchronize final chart and report closure candidate
</commit_message>
<xml_diff>
--- a/docs/research/integrated-product-106/Experience/cases/HOME-12/HOME-12_Evidence_Workbook.xlsx
+++ b/docs/research/integrated-product-106/Experience/cases/HOME-12/HOME-12_Evidence_Workbook.xlsx
@@ -387,7 +387,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t>None</a:t>
+                <a:t/>
               </a:r>
               <a:endParaRPr sz="1100" b="0">
                 <a:latin typeface="Archivo"/>
@@ -438,7 +438,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr sz="1100" b="0">
               <a:latin typeface="Archivo"/>
@@ -466,7 +466,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr sz="1100" b="0">
               <a:latin typeface="Archivo"/>
@@ -546,7 +546,7 @@
                 </a:defRPr>
               </a:pPr>
               <a:r>
-                <a:t>None</a:t>
+                <a:t/>
               </a:r>
               <a:endParaRPr sz="1100" b="0">
                 <a:latin typeface="Archivo"/>
@@ -597,7 +597,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr sz="1100" b="0">
               <a:latin typeface="Archivo"/>
@@ -625,7 +625,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t>None</a:t>
+              <a:t/>
             </a:r>
             <a:endParaRPr sz="1100" b="0">
               <a:latin typeface="Archivo"/>

</xml_diff>